<commit_message>
initial commit of app
</commit_message>
<xml_diff>
--- a/household_budget_template.xlsx
+++ b/household_budget_template.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -728,12 +728,14 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="8" t="n"/>
+        <v>2800</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>17</v>
+      </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Fill in</t>
+          <t>Joint account — TLP RE Client Acc (letting agent), confirmed 12/12 months</t>
         </is>
       </c>
     </row>
@@ -754,7 +756,7 @@
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>e.g. service charge, maintenance</t>
+          <t>Council Tax is paid as an annual lump sum — see Upcoming Expenses (~£1,020, due ~Apr)</t>
         </is>
       </c>
     </row>
@@ -795,10 +797,16 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>64</v>
-      </c>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="9" t="inlineStr"/>
+        <v>68.76000000000001</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>E.ON Next DD, Joint account — actual avg £68.76 (range £62-76), was budgeted £64</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -812,10 +820,16 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="9" t="inlineStr"/>
+        <v>20.56</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Community Fibre DD, Joint account — confirmed, very stable</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -832,7 +846,11 @@
         <v>23</v>
       </c>
       <c r="D22" s="8" t="n"/>
-      <c r="E22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Not found in reviewed statements — verify still active / correct amount</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -846,10 +864,16 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="9" t="inlineStr"/>
+        <v>23.02</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Urban Jungle DD, Joint account — renewed from £15.02 to £23.02/mo in Apr 2026</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -884,14 +908,20 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Car expenses</t>
+          <t>Car tax — B355RHC (DVLA)</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>142</v>
-      </c>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="9" t="inlineStr"/>
+        <v>31.5</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Personal HSBC DD — was bundled into "Car expenses 142"</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -901,73 +931,89 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Car expenses</t>
+          <t>Car tax — C800BWR (DVLA)</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="9" t="inlineStr"/>
+        <v>32.81</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Personal HSBC DD — second car, was bundled into "Car expenses 142"</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Car insurance (Elephant)</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>77.53</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Personal HSBC DD — was bundled into "Car expenses 142"</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>102.54</v>
+      </c>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Variable card spend, Joint account — avg per active month, not a fixed DD (was "Car expenses 100")</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Total Transport</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="12">
-        <f>SUM(C27:C28)</f>
-        <v/>
-      </c>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="12">
+        <f>SUM(C27:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>SUBSCRIPTIONS</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Subscriptions</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Spotify</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Subscriptions</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Netflix</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="9" t="inlineStr"/>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -977,14 +1023,20 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="D34" s="8" t="n"/>
-      <c r="E34" s="9" t="inlineStr"/>
+        <v>17.66</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Personal Monzo — confirmed, day varies 1-11</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -994,14 +1046,20 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Netflix</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D35" s="8" t="n"/>
-      <c r="E35" s="9" t="inlineStr"/>
+        <v>5.99</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Joint account — confirmed exact</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1011,14 +1069,20 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Amazon Prime</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D36" s="8" t="n"/>
-      <c r="E36" s="9" t="inlineStr"/>
+        <v>8.99</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Amex — confirmed exact</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1028,14 +1092,18 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>TV licence</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D37" s="8" t="n"/>
-      <c r="E37" s="9" t="inlineStr"/>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Not confirmed monthly — only a one-off £53.99 Amex charge seen; verify what this is</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1045,150 +1113,206 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Not found in reviewed statements — verify still active</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>TV licence</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>TV Licensing DD, Joint account — actual is £36, was budgeted £15; only seen Jun &amp; Jul (may be a 10-month DD scheme)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
           <t>AWS</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D38" s="8" t="n"/>
-      <c r="E38" s="9" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Total Subscriptions</t>
-        </is>
-      </c>
-      <c r="B39" s="11" t="n"/>
-      <c r="C39" s="12">
-        <f>SUM(C32:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="11" t="n"/>
-      <c r="E39" s="11" t="n"/>
+      <c r="C40" s="7" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Usage-based, Personal Monzo — avg £23.53 (range ~£14-33), varies month to month, was budgeted £5</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>PERSONAL &amp; OTHER</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Claude.ai</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>New — Amex, confirmed 3/3 months, not in original list</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Voxi (Vodafone) mobile</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>New — Personal HSBC, variable £4.80-16, present every month, not in original list</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Total Subscriptions</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="12">
+        <f>SUM(C34:C42)</f>
+        <v/>
+      </c>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PERSONAL &amp; OTHER</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Nathan</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n">
+      <c r="C46" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="D42" s="8" t="n"/>
-      <c r="E42" s="9" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>Swimming</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="D43" s="8" t="n"/>
-      <c r="E43" s="9" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Total Personal &amp; Other</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="n"/>
-      <c r="C44" s="12">
-        <f>SUM(C42:C43)</f>
-        <v/>
-      </c>
-      <c r="D44" s="11" t="n"/>
-      <c r="E44" s="11" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>SAVINGS &amp; INVESTMENTS</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="5" t="n"/>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="5" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Not found in reviewed statements — verify (may be paid via cash/another account)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Monthly savings contribution</t>
+          <t>Swimming</t>
         </is>
       </c>
       <c r="C47" s="7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D47" s="8" t="n"/>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Fill in</t>
+          <t>Not found in reviewed statements — verify (may be paid via cash/another account)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Investments</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Monthly investment contribution</t>
+          <t>The Riders Hub</t>
         </is>
       </c>
       <c r="C48" s="7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D48" s="8" t="n"/>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Fill in</t>
+          <t>Low confidence — appears sporadically on personal HSBC &amp; Monzo, possibly a lesson/hobby subscription; verify</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Total Savings &amp; Investments</t>
+          <t>Total Personal &amp; Other</t>
         </is>
       </c>
       <c r="B49" s="11" t="n"/>
       <c r="C49" s="12">
-        <f>SUM(C47:C48)</f>
+        <f>SUM(C46:C48)</f>
         <v/>
       </c>
       <c r="D49" s="11" t="n"/>
@@ -1197,7 +1321,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>SUMMARY</t>
+          <t>SAVINGS &amp; INVESTMENTS</t>
         </is>
       </c>
       <c r="B51" s="5" t="n"/>
@@ -1206,50 +1330,117 @@
       <c r="E51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>Total Income</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="14">
-        <f>C12</f>
-        <v/>
-      </c>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="6" t="n"/>
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Monthly savings contribution</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Fill in</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>Total Outgoings (Housing + Expenses + Savings)</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="14">
-        <f>C17+C24+C29+C39+C44+C49</f>
-        <v/>
-      </c>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Monthly investment contribution</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Fill in</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="15" t="inlineStr">
-        <is>
-          <t>Net Remaining</t>
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Total Savings &amp; Investments</t>
         </is>
       </c>
       <c r="B54" s="11" t="n"/>
-      <c r="C54" s="16">
-        <f>C12-C53</f>
+      <c r="C54" s="12">
+        <f>SUM(C52:C53)</f>
         <v/>
       </c>
       <c r="D54" s="11" t="n"/>
       <c r="E54" s="11" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="14">
+        <f>C12</f>
+        <v/>
+      </c>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Total Outgoings (Housing + Expenses + Savings)</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="14">
+        <f>C17+C24+C31+C43+C49+C54</f>
+        <v/>
+      </c>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Net Remaining</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="16">
+        <f>C12-C58</f>
+        <v/>
+      </c>
+      <c r="D59" s="11" t="n"/>
+      <c r="E59" s="11" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D6 D7 D8 D9 D10 D11 D15 D16 D20 D21 D22 D23 D27 D28 D32 D33 D34 D35 D36 D37 D38 D42 D43 D47 D48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid day" error="Enter a day of month between 1 and 31, or leave blank." type="whole" operator="between">
+    <dataValidation sqref="D6 D7 D8 D9 D10 D11 D15 D16 D20 D21 D22 D23 D27 D28 D29 D30 D34 D35 D36 D37 D38 D39 D40 D41 D42 D46 D47 D48 D52 D53" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid day" error="Enter a day of month between 1 and 31, or leave blank." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>31</formula2>
     </dataValidation>
@@ -1525,16 +1716,40 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="18" t="n"/>
+      <c r="A5" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Thames Water (6-monthly)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Recurs ~every 6 months; last seen ~Apr 2026 (~£186-190), Joint account</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n"/>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="18" t="n"/>
+      <c r="A6" s="17" t="n">
+        <v>46504</v>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Council Tax (Wandsworth) — annual</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>1020.35</v>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Paid as an annual lump sum from the Joint account; may increase with rate changes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="n"/>
@@ -1998,11 +2213,11 @@
         <v/>
       </c>
       <c r="B7" s="14">
-        <f>IF(A7="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,1))</f>
+        <f>IF(A7="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,1))</f>
         <v/>
       </c>
       <c r="C7" s="14">
-        <f>IF(A7="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,1))</f>
+        <f>IF(A7="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,1))</f>
         <v/>
       </c>
       <c r="D7" s="14">
@@ -2033,11 +2248,11 @@
         <v/>
       </c>
       <c r="B8" s="14">
-        <f>IF(A8="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,2))</f>
+        <f>IF(A8="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,2))</f>
         <v/>
       </c>
       <c r="C8" s="14">
-        <f>IF(A8="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,2))</f>
+        <f>IF(A8="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,2))</f>
         <v/>
       </c>
       <c r="D8" s="14">
@@ -2068,11 +2283,11 @@
         <v/>
       </c>
       <c r="B9" s="14">
-        <f>IF(A9="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,3))</f>
+        <f>IF(A9="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,3))</f>
         <v/>
       </c>
       <c r="C9" s="14">
-        <f>IF(A9="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,3))</f>
+        <f>IF(A9="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,3))</f>
         <v/>
       </c>
       <c r="D9" s="14">
@@ -2103,11 +2318,11 @@
         <v/>
       </c>
       <c r="B10" s="14">
-        <f>IF(A10="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,4))</f>
+        <f>IF(A10="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,4))</f>
         <v/>
       </c>
       <c r="C10" s="14">
-        <f>IF(A10="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,4))</f>
+        <f>IF(A10="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,4))</f>
         <v/>
       </c>
       <c r="D10" s="14">
@@ -2138,11 +2353,11 @@
         <v/>
       </c>
       <c r="B11" s="14">
-        <f>IF(A11="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,5))</f>
+        <f>IF(A11="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,5))</f>
         <v/>
       </c>
       <c r="C11" s="14">
-        <f>IF(A11="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,5))</f>
+        <f>IF(A11="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,5))</f>
         <v/>
       </c>
       <c r="D11" s="14">
@@ -2173,11 +2388,11 @@
         <v/>
       </c>
       <c r="B12" s="14">
-        <f>IF(A12="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,6))</f>
+        <f>IF(A12="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,6))</f>
         <v/>
       </c>
       <c r="C12" s="14">
-        <f>IF(A12="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,6))</f>
+        <f>IF(A12="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,6))</f>
         <v/>
       </c>
       <c r="D12" s="14">
@@ -2208,11 +2423,11 @@
         <v/>
       </c>
       <c r="B13" s="14">
-        <f>IF(A13="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,7))</f>
+        <f>IF(A13="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,7))</f>
         <v/>
       </c>
       <c r="C13" s="14">
-        <f>IF(A13="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,7))</f>
+        <f>IF(A13="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,7))</f>
         <v/>
       </c>
       <c r="D13" s="14">
@@ -2243,11 +2458,11 @@
         <v/>
       </c>
       <c r="B14" s="14">
-        <f>IF(A14="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,8))</f>
+        <f>IF(A14="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,8))</f>
         <v/>
       </c>
       <c r="C14" s="14">
-        <f>IF(A14="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,8))</f>
+        <f>IF(A14="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,8))</f>
         <v/>
       </c>
       <c r="D14" s="14">
@@ -2278,11 +2493,11 @@
         <v/>
       </c>
       <c r="B15" s="14">
-        <f>IF(A15="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,9))</f>
+        <f>IF(A15="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,9))</f>
         <v/>
       </c>
       <c r="C15" s="14">
-        <f>IF(A15="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,9))</f>
+        <f>IF(A15="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,9))</f>
         <v/>
       </c>
       <c r="D15" s="14">
@@ -2313,11 +2528,11 @@
         <v/>
       </c>
       <c r="B16" s="14">
-        <f>IF(A16="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,10))</f>
+        <f>IF(A16="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,10))</f>
         <v/>
       </c>
       <c r="C16" s="14">
-        <f>IF(A16="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,10))</f>
+        <f>IF(A16="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,10))</f>
         <v/>
       </c>
       <c r="D16" s="14">
@@ -2348,11 +2563,11 @@
         <v/>
       </c>
       <c r="B17" s="14">
-        <f>IF(A17="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,11))</f>
+        <f>IF(A17="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,11))</f>
         <v/>
       </c>
       <c r="C17" s="14">
-        <f>IF(A17="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,11))</f>
+        <f>IF(A17="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,11))</f>
         <v/>
       </c>
       <c r="D17" s="14">
@@ -2383,11 +2598,11 @@
         <v/>
       </c>
       <c r="B18" s="14">
-        <f>IF(A18="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,12))</f>
+        <f>IF(A18="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,12))</f>
         <v/>
       </c>
       <c r="C18" s="14">
-        <f>IF(A18="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,12))</f>
+        <f>IF(A18="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,12))</f>
         <v/>
       </c>
       <c r="D18" s="14">
@@ -2418,11 +2633,11 @@
         <v/>
       </c>
       <c r="B19" s="14">
-        <f>IF(A19="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,13))</f>
+        <f>IF(A19="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,13))</f>
         <v/>
       </c>
       <c r="C19" s="14">
-        <f>IF(A19="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,13))</f>
+        <f>IF(A19="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,13))</f>
         <v/>
       </c>
       <c r="D19" s="14">
@@ -2453,11 +2668,11 @@
         <v/>
       </c>
       <c r="B20" s="14">
-        <f>IF(A20="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,14))</f>
+        <f>IF(A20="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,14))</f>
         <v/>
       </c>
       <c r="C20" s="14">
-        <f>IF(A20="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,14))</f>
+        <f>IF(A20="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,14))</f>
         <v/>
       </c>
       <c r="D20" s="14">
@@ -2488,11 +2703,11 @@
         <v/>
       </c>
       <c r="B21" s="14">
-        <f>IF(A21="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,15))</f>
+        <f>IF(A21="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,15))</f>
         <v/>
       </c>
       <c r="C21" s="14">
-        <f>IF(A21="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,15))</f>
+        <f>IF(A21="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,15))</f>
         <v/>
       </c>
       <c r="D21" s="14">
@@ -2523,11 +2738,11 @@
         <v/>
       </c>
       <c r="B22" s="14">
-        <f>IF(A22="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,16))</f>
+        <f>IF(A22="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,16))</f>
         <v/>
       </c>
       <c r="C22" s="14">
-        <f>IF(A22="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,16))</f>
+        <f>IF(A22="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,16))</f>
         <v/>
       </c>
       <c r="D22" s="14">
@@ -2558,11 +2773,11 @@
         <v/>
       </c>
       <c r="B23" s="14">
-        <f>IF(A23="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,17))</f>
+        <f>IF(A23="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,17))</f>
         <v/>
       </c>
       <c r="C23" s="14">
-        <f>IF(A23="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,17))</f>
+        <f>IF(A23="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,17))</f>
         <v/>
       </c>
       <c r="D23" s="14">
@@ -2593,11 +2808,11 @@
         <v/>
       </c>
       <c r="B24" s="14">
-        <f>IF(A24="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,18))</f>
+        <f>IF(A24="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,18))</f>
         <v/>
       </c>
       <c r="C24" s="14">
-        <f>IF(A24="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,18))</f>
+        <f>IF(A24="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,18))</f>
         <v/>
       </c>
       <c r="D24" s="14">
@@ -2628,11 +2843,11 @@
         <v/>
       </c>
       <c r="B25" s="14">
-        <f>IF(A25="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,19))</f>
+        <f>IF(A25="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,19))</f>
         <v/>
       </c>
       <c r="C25" s="14">
-        <f>IF(A25="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,19))</f>
+        <f>IF(A25="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,19))</f>
         <v/>
       </c>
       <c r="D25" s="14">
@@ -2663,11 +2878,11 @@
         <v/>
       </c>
       <c r="B26" s="14">
-        <f>IF(A26="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,20))</f>
+        <f>IF(A26="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,20))</f>
         <v/>
       </c>
       <c r="C26" s="14">
-        <f>IF(A26="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,20))</f>
+        <f>IF(A26="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,20))</f>
         <v/>
       </c>
       <c r="D26" s="14">
@@ -2698,11 +2913,11 @@
         <v/>
       </c>
       <c r="B27" s="14">
-        <f>IF(A27="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,21))</f>
+        <f>IF(A27="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,21))</f>
         <v/>
       </c>
       <c r="C27" s="14">
-        <f>IF(A27="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,21))</f>
+        <f>IF(A27="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,21))</f>
         <v/>
       </c>
       <c r="D27" s="14">
@@ -2733,11 +2948,11 @@
         <v/>
       </c>
       <c r="B28" s="14">
-        <f>IF(A28="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,22))</f>
+        <f>IF(A28="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,22))</f>
         <v/>
       </c>
       <c r="C28" s="14">
-        <f>IF(A28="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,22))</f>
+        <f>IF(A28="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,22))</f>
         <v/>
       </c>
       <c r="D28" s="14">
@@ -2768,11 +2983,11 @@
         <v/>
       </c>
       <c r="B29" s="14">
-        <f>IF(A29="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,23))</f>
+        <f>IF(A29="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,23))</f>
         <v/>
       </c>
       <c r="C29" s="14">
-        <f>IF(A29="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,23))</f>
+        <f>IF(A29="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,23))</f>
         <v/>
       </c>
       <c r="D29" s="14">
@@ -2803,11 +3018,11 @@
         <v/>
       </c>
       <c r="B30" s="14">
-        <f>IF(A30="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,24))</f>
+        <f>IF(A30="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,24))</f>
         <v/>
       </c>
       <c r="C30" s="14">
-        <f>IF(A30="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,24))</f>
+        <f>IF(A30="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,24))</f>
         <v/>
       </c>
       <c r="D30" s="14">
@@ -2838,11 +3053,11 @@
         <v/>
       </c>
       <c r="B31" s="14">
-        <f>IF(A31="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,25))</f>
+        <f>IF(A31="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,25))</f>
         <v/>
       </c>
       <c r="C31" s="14">
-        <f>IF(A31="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,25))</f>
+        <f>IF(A31="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,25))</f>
         <v/>
       </c>
       <c r="D31" s="14">
@@ -2873,11 +3088,11 @@
         <v/>
       </c>
       <c r="B32" s="14">
-        <f>IF(A32="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,26))</f>
+        <f>IF(A32="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,26))</f>
         <v/>
       </c>
       <c r="C32" s="14">
-        <f>IF(A32="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,26))</f>
+        <f>IF(A32="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,26))</f>
         <v/>
       </c>
       <c r="D32" s="14">
@@ -2908,11 +3123,11 @@
         <v/>
       </c>
       <c r="B33" s="14">
-        <f>IF(A33="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,27))</f>
+        <f>IF(A33="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,27))</f>
         <v/>
       </c>
       <c r="C33" s="14">
-        <f>IF(A33="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,27))</f>
+        <f>IF(A33="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,27))</f>
         <v/>
       </c>
       <c r="D33" s="14">
@@ -2943,11 +3158,11 @@
         <v/>
       </c>
       <c r="B34" s="14">
-        <f>IF(A34="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,28))</f>
+        <f>IF(A34="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,28))</f>
         <v/>
       </c>
       <c r="C34" s="14">
-        <f>IF(A34="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,28))</f>
+        <f>IF(A34="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,28))</f>
         <v/>
       </c>
       <c r="D34" s="14">
@@ -2978,11 +3193,11 @@
         <v/>
       </c>
       <c r="B35" s="14">
-        <f>IF(A35="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,29))</f>
+        <f>IF(A35="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,29))</f>
         <v/>
       </c>
       <c r="C35" s="14">
-        <f>IF(A35="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,29))</f>
+        <f>IF(A35="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,29))</f>
         <v/>
       </c>
       <c r="D35" s="14">
@@ -3013,11 +3228,11 @@
         <v/>
       </c>
       <c r="B36" s="14">
-        <f>IF(A36="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,30))</f>
+        <f>IF(A36="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,30))</f>
         <v/>
       </c>
       <c r="C36" s="14">
-        <f>IF(A36="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,30))</f>
+        <f>IF(A36="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,30))</f>
         <v/>
       </c>
       <c r="D36" s="14">
@@ -3048,11 +3263,11 @@
         <v/>
       </c>
       <c r="B37" s="14">
-        <f>IF(A37="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"Income",Budget!$D$5:$D$56,31))</f>
+        <f>IF(A37="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"Income",Budget!$D$5:$D$61,31))</f>
         <v/>
       </c>
       <c r="C37" s="14">
-        <f>IF(A37="","",SUMIFS(Budget!$C$5:$C$56,Budget!$A$5:$A$56,"&lt;&gt;Income",Budget!$D$5:$D$56,31))</f>
+        <f>IF(A37="","",SUMIFS(Budget!$C$5:$C$61,Budget!$A$5:$A$61,"&lt;&gt;Income",Budget!$D$5:$D$61,31))</f>
         <v/>
       </c>
       <c r="D37" s="14">

</xml_diff>